<commit_message>
License under PolyForm Noncommercial 1.0.0 and CC BY-NC 4.0
Code under the PolyForm Noncommercial License 1.0.0 (LICENSE.md, with
Required Notice lines; SPDX headers in source files). Documents,
templates and data under CC BY-NC 4.0 (LICENSE-docs.txt; licence note in
the template's Read me sheet). README sets out which files fall under
which licence; CITATION.cff records both. The engine's start-up message
states the licence. Third-party notices updated.
</commit_message>
<xml_diff>
--- a/templates/JAF_template_illustrative_INVENTED_STATES.xlsx
+++ b/templates/JAF_template_illustrative_INVENTED_STATES.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A58"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -717,138 +717,169 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Data for testing the model (optional; build plan s 14)</t>
+          <t>Licence</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>The sheets Episodes, Data, Measurement, Estimation and Hypotheses hold an empirical design. They are needed only</t>
+          <t>This template is part of JAF Rule Bench, Copyright (c) 2026 Wen Yi LEONG, and is licensed under the Creative</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>to estimate the model's behavioural parameters from observed facts and to test its predictions (the 'Test against</t>
+          <t>Commons Attribution-NonCommercial 4.0 International licence (CC BY-NC 4.0):</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>data' tab). Leave them empty to use the tool as before.</t>
+          <t>https://creativecommons.org/licenses/by-nc/4.0/. The entries you add to it are your own.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>- Episodes: versions of the coded law to compare. 'baseline' is the coded world as loaded. Each other episode is a</t>
-        </is>
-      </c>
+      <c r="A43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  list of changes, one per row: the jurisdiction code (or 'settings'), the field to change and its new value.</t>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Data for testing the model (optional; build plan s 14)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A single reform (for example India's 2022 regime) is one episode that changes one state's rate and collection.</t>
+          <t>The sheets Episodes, Data, Measurement, Estimation and Hypotheses hold an empirical design. They are needed only</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Staggered adoption of automatic exchange (for example the CARF waves) is one episode per wave, each setting the</t>
+          <t>to estimate the model's behavioural parameters from observed facts and to test its predictions (the 'Test against</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">  scenario year (and, if needed, a state's first year of exchange).</t>
+          <t>data' tab). Leave them empty to use the tool as before.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>- Data: one row per observed fact. Choose the quantity from the drop-down list (the Quantities sheet explains what</t>
+          <t>- Episodes: versions of the coded law to compare. 'baseline' is the coded world as loaded. Each other episode is a</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">  each measures and how data record it), the jurisdiction, the episode and, for a change, the episode it is</t>
+          <t xml:space="preserve">  list of changes, one per row: the jurisdiction code (or 'settings'), the field to change and its new value.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  compared with. Give the standard error of the value: it says how far the value could be off, and the fit is</t>
+          <t xml:space="preserve">  A single reform (for example India's 2022 regime) is one episode that changes one state's rate and collection.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">  weighted by it. Mark each row target (used to estimate) or holdout (kept back to test the predictions).</t>
+          <t xml:space="preserve">  Staggered adoption of automatic exchange (for example the CARF waves) is one episode per wave, each setting the</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Leave values blank, fill everything else, and freeze the design on the tab before looking at the data: that</t>
+          <t xml:space="preserve">  scenario year (and, if needed, a state's first year of exchange).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  is the pre-registration.</t>
+          <t>- Data: one row per observed fact. Choose the quantity from the drop-down list (the Quantities sheet explains what</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>- Measurement: for exchange data, the share of reported volume that is wash trading at exchanges based in each</t>
+          <t xml:space="preserve">  each measures and how data record it), the jurisdiction, the episode and, for a change, the episode it is</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  place, and genuine turnover relative to elsewhere (1 if unknown). Volume-based quantities are adjusted for both.</t>
+          <t xml:space="preserve">  compared with. Give the standard error of the value: it says how far the value could be off, and the fit is</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>- Estimation: which behavioural parameters to estimate (free = yes, with a start value and bounds) and which to fix</t>
+          <t xml:space="preserve">  weighted by it. Mark each row target (used to estimate) or holdout (kept back to test the predictions).</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">  by judgement (free = no, with a value and, optionally, a plausible range used to widen prediction bands).</t>
+          <t xml:space="preserve">  Leave values blank, fill everything else, and freeze the design on the tab before looking at the data: that</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  is the pre-registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>- Measurement: for exchange data, the share of reported volume that is wash trading at exchanges based in each</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  place, and genuine turnover relative to elsewhere (1 if unknown). Volume-based quantities are adjusted for both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>- Estimation: which behavioural parameters to estimate (free = yes, with a start value and bounds) and which to fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  by judgement (free = no, with a value and, optionally, a plausible range used to widen prediction bands).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>- Hypotheses: the claims the data are to test, and what result would support or refute each.</t>
         </is>

</xml_diff>